<commit_message>
updated seismic in-class exercise
</commit_message>
<xml_diff>
--- a/docs/unit2/09_seismic/files/seismic_johnson_res_KEY.xlsx
+++ b/docs/unit2/09_seismic/files/seismic_johnson_res_KEY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/temp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E49ADBC0-F2C9-2948-A83D-E102434327CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7532AD6-6276-C04E-99DC-B78CDE0C8CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6460" yWindow="5000" windowWidth="30840" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1700" yWindow="5700" windowWidth="30840" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -7887,10 +7887,10 @@
         <v>34</v>
       </c>
       <c r="E9" s="3">
-        <v>100</v>
+        <v>1400</v>
       </c>
       <c r="F9" s="3">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -7937,10 +7937,10 @@
         <v>34</v>
       </c>
       <c r="E10" s="3">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="F10" s="3">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -7987,10 +7987,10 @@
         <v>34</v>
       </c>
       <c r="E11" s="3">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="F11" s="3">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -9942,20 +9942,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -9972,6 +9958,20 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>